<commit_message>
chore: update RPS hash values [2026-09-13 07:07 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1363,14 +1363,10 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>8c759814e1f9f1e275910795724f2ebba8f9d96da3b42cd0b7049a4fa4632e0e</t>
-        </is>
-      </c>
-      <c r="C87" s="8" t="inlineStr">
-        <is>
           <t>ef692a6abff59e8b699d3e69d6974057ed5a5cc33d9d7a8f1d43f9f6342941f4</t>
         </is>
       </c>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1435,7 +1431,11 @@
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
-      <c r="C92" s="3" t="n"/>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
+          <t>ef692a6abff59e8b699d3e69d6974057ed5a5cc33d9d7a8f1d43f9f6342941f4</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -2424,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F123"/>
+  <dimension ref="A1:F124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5391,6 +5391,30 @@
         </is>
       </c>
     </row>
+    <row r="124">
+      <c r="A124" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-13 07:06:21</t>
+        </is>
+      </c>
+      <c r="B124" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C124" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D124" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E124" s="5" t="n">
+        <v>173</v>
+      </c>
+      <c r="F124" s="5" t="inlineStr">
+        <is>
+          <t>PRM_AK_DHSS_EPL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-09-14 07:40 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,7 +1366,11 @@
           <t>ef692a6abff59e8b699d3e69d6974057ed5a5cc33d9d7a8f1d43f9f6342941f4</t>
         </is>
       </c>
-      <c r="C87" s="3" t="n"/>
+      <c r="C87" s="9" t="inlineStr">
+        <is>
+          <t>ef692a6abff59e8b699d3e69d6974057ed5a5cc33d9d7a8f1d43f9f6342941f4</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1428,12 +1432,12 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
+          <t>ef692a6abff59e8b699d3e69d6974057ed5a5cc33d9d7a8f1d43f9f6342941f4</t>
+        </is>
+      </c>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
-        </is>
-      </c>
-      <c r="C92" s="8" t="inlineStr">
-        <is>
-          <t>ef692a6abff59e8b699d3e69d6974057ed5a5cc33d9d7a8f1d43f9f6342941f4</t>
         </is>
       </c>
     </row>
@@ -1941,11 +1945,7 @@
           <t>eb691cf34a1437fa12fdf43cc9e8b331a8f8ade2c53450c3e4a520d5d1b259db</t>
         </is>
       </c>
-      <c r="C134" s="9" t="inlineStr">
-        <is>
-          <t>eb691cf34a1437fa12fdf43cc9e8b331a8f8ade2c53450c3e4a520d5d1b259db</t>
-        </is>
-      </c>
+      <c r="C134" s="3" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -2424,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F124"/>
+  <dimension ref="A1:F125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5415,6 +5415,30 @@
         </is>
       </c>
     </row>
+    <row r="125">
+      <c r="A125" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-14 07:29:48</t>
+        </is>
+      </c>
+      <c r="B125" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C125" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D125" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E125" s="6" t="n">
+        <v>173</v>
+      </c>
+      <c r="F125" s="6" t="inlineStr">
+        <is>
+          <t>PRM_AK_DHSS_EPL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-09-15 07:17 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,11 +1366,7 @@
           <t>ef692a6abff59e8b699d3e69d6974057ed5a5cc33d9d7a8f1d43f9f6342941f4</t>
         </is>
       </c>
-      <c r="C87" s="9" t="inlineStr">
-        <is>
-          <t>ef692a6abff59e8b699d3e69d6974057ed5a5cc33d9d7a8f1d43f9f6342941f4</t>
-        </is>
-      </c>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1432,12 +1428,12 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
+          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
+        </is>
+      </c>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
           <t>ef692a6abff59e8b699d3e69d6974057ed5a5cc33d9d7a8f1d43f9f6342941f4</t>
-        </is>
-      </c>
-      <c r="C92" s="8" t="inlineStr">
-        <is>
-          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
     </row>
@@ -2424,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F125"/>
+  <dimension ref="A1:F126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5439,6 +5435,30 @@
         </is>
       </c>
     </row>
+    <row r="126">
+      <c r="A126" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-15 07:06:54</t>
+        </is>
+      </c>
+      <c r="B126" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C126" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D126" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E126" s="5" t="n">
+        <v>174</v>
+      </c>
+      <c r="F126" s="5" t="inlineStr">
+        <is>
+          <t>PRM_AK_DHSS_EPL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-09-16 07:17 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,7 +1366,11 @@
           <t>ef692a6abff59e8b699d3e69d6974057ed5a5cc33d9d7a8f1d43f9f6342941f4</t>
         </is>
       </c>
-      <c r="C87" s="3" t="n"/>
+      <c r="C87" s="9" t="inlineStr">
+        <is>
+          <t>ef692a6abff59e8b699d3e69d6974057ed5a5cc33d9d7a8f1d43f9f6342941f4</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1428,14 +1432,10 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
-        </is>
-      </c>
-      <c r="C92" s="8" t="inlineStr">
-        <is>
           <t>ef692a6abff59e8b699d3e69d6974057ed5a5cc33d9d7a8f1d43f9f6342941f4</t>
         </is>
       </c>
+      <c r="C92" s="3" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -2420,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F126"/>
+  <dimension ref="A1:F127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5459,6 +5459,30 @@
         </is>
       </c>
     </row>
+    <row r="127">
+      <c r="A127" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:07:17</t>
+        </is>
+      </c>
+      <c r="B127" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C127" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D127" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E127" s="6" t="n">
+        <v>174</v>
+      </c>
+      <c r="F127" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-09-17 07:15 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,11 +1366,7 @@
           <t>ef692a6abff59e8b699d3e69d6974057ed5a5cc33d9d7a8f1d43f9f6342941f4</t>
         </is>
       </c>
-      <c r="C87" s="9" t="inlineStr">
-        <is>
-          <t>ef692a6abff59e8b699d3e69d6974057ed5a5cc33d9d7a8f1d43f9f6342941f4</t>
-        </is>
-      </c>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1492,7 +1488,11 @@
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
-      <c r="C97" s="3" t="n"/>
+      <c r="C97" s="8" t="inlineStr">
+        <is>
+          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2420,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F127"/>
+  <dimension ref="A1:F128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5483,6 +5483,30 @@
         </is>
       </c>
     </row>
+    <row r="128">
+      <c r="A128" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-17 07:05:43</t>
+        </is>
+      </c>
+      <c r="B128" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C128" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D128" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E128" s="5" t="n">
+        <v>174</v>
+      </c>
+      <c r="F128" s="5" t="inlineStr">
+        <is>
+          <t>PRM_DC_DDS_PSL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-09-18 07:00 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,7 +1366,11 @@
           <t>ef692a6abff59e8b699d3e69d6974057ed5a5cc33d9d7a8f1d43f9f6342941f4</t>
         </is>
       </c>
-      <c r="C87" s="3" t="n"/>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>b7b891194dc167ef9afbe42ce2a129f412263694610b951b3bf269136821f30c</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1485,14 +1489,10 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
-        </is>
-      </c>
-      <c r="C97" s="8" t="inlineStr">
-        <is>
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
+      <c r="C97" s="3" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -1941,7 +1941,11 @@
           <t>eb691cf34a1437fa12fdf43cc9e8b331a8f8ade2c53450c3e4a520d5d1b259db</t>
         </is>
       </c>
-      <c r="C134" s="3" t="n"/>
+      <c r="C134" s="8" t="inlineStr">
+        <is>
+          <t>d396b80a78fcbfbb48a9a68e42d5229d71a947bca970a9ccb07ba181250ab2d7</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -2257,7 +2261,11 @@
           <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
         </is>
       </c>
-      <c r="C162" s="3" t="n"/>
+      <c r="C162" s="8" t="inlineStr">
+        <is>
+          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2420,7 +2428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F128"/>
+  <dimension ref="A1:F129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5507,6 +5515,30 @@
         </is>
       </c>
     </row>
+    <row r="129">
+      <c r="A129" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-18 06:59:06</t>
+        </is>
+      </c>
+      <c r="B129" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C129" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D129" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E129" s="6" t="n">
+        <v>172</v>
+      </c>
+      <c r="F129" s="6" t="inlineStr">
+        <is>
+          <t>OIG_MOST_WANTED, PRM_WI_DOT_DSIC, US_DOT_MOST_WANTED</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-09-19 07:08 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1363,12 +1363,12 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>ef692a6abff59e8b699d3e69d6974057ed5a5cc33d9d7a8f1d43f9f6342941f4</t>
+          <t>b7b891194dc167ef9afbe42ce2a129f412263694610b951b3bf269136821f30c</t>
         </is>
       </c>
       <c r="C87" s="8" t="inlineStr">
         <is>
-          <t>b7b891194dc167ef9afbe42ce2a129f412263694610b951b3bf269136821f30c</t>
+          <t>2f510140dc68e0c74c5ac10571c7237154c98f6810ad4b314bd1b1fedd391d49</t>
         </is>
       </c>
     </row>
@@ -1938,14 +1938,10 @@
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>eb691cf34a1437fa12fdf43cc9e8b331a8f8ade2c53450c3e4a520d5d1b259db</t>
-        </is>
-      </c>
-      <c r="C134" s="8" t="inlineStr">
-        <is>
           <t>d396b80a78fcbfbb48a9a68e42d5229d71a947bca970a9ccb07ba181250ab2d7</t>
         </is>
       </c>
+      <c r="C134" s="3" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -2258,14 +2254,10 @@
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
-        </is>
-      </c>
-      <c r="C162" s="8" t="inlineStr">
-        <is>
           <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
         </is>
       </c>
+      <c r="C162" s="3" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2428,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F129"/>
+  <dimension ref="A1:F130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5539,6 +5531,30 @@
         </is>
       </c>
     </row>
+    <row r="130">
+      <c r="A130" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-19 06:58:03</t>
+        </is>
+      </c>
+      <c r="B130" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C130" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D130" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E130" s="5" t="n">
+        <v>174</v>
+      </c>
+      <c r="F130" s="5" t="inlineStr">
+        <is>
+          <t>OIG_MOST_WANTED</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-09-20 07:33 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1363,10 +1363,10 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>b7b891194dc167ef9afbe42ce2a129f412263694610b951b3bf269136821f30c</t>
-        </is>
-      </c>
-      <c r="C87" s="8" t="inlineStr">
+          <t>2f510140dc68e0c74c5ac10571c7237154c98f6810ad4b314bd1b1fedd391d49</t>
+        </is>
+      </c>
+      <c r="C87" s="9" t="inlineStr">
         <is>
           <t>2f510140dc68e0c74c5ac10571c7237154c98f6810ad4b314bd1b1fedd391d49</t>
         </is>
@@ -2420,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F130"/>
+  <dimension ref="A1:F131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5555,6 +5555,30 @@
         </is>
       </c>
     </row>
+    <row r="131">
+      <c r="A131" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-20 07:23:09</t>
+        </is>
+      </c>
+      <c r="B131" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C131" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D131" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E131" s="6" t="n">
+        <v>174</v>
+      </c>
+      <c r="F131" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-09-21 07:35 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1941,7 +1941,11 @@
           <t>d396b80a78fcbfbb48a9a68e42d5229d71a947bca970a9ccb07ba181250ab2d7</t>
         </is>
       </c>
-      <c r="C134" s="3" t="n"/>
+      <c r="C134" s="9" t="inlineStr">
+        <is>
+          <t>d396b80a78fcbfbb48a9a68e42d5229d71a947bca970a9ccb07ba181250ab2d7</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -2420,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F131"/>
+  <dimension ref="A1:F132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5579,6 +5583,30 @@
         </is>
       </c>
     </row>
+    <row r="132">
+      <c r="A132" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-21 07:33:40</t>
+        </is>
+      </c>
+      <c r="B132" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C132" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D132" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E132" s="5" t="n">
+        <v>173</v>
+      </c>
+      <c r="F132" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-09-22 07:21 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -2424,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F132"/>
+  <dimension ref="A1:F133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5607,6 +5607,30 @@
         </is>
       </c>
     </row>
+    <row r="133">
+      <c r="A133" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-22 07:13:11</t>
+        </is>
+      </c>
+      <c r="B133" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C133" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D133" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E133" s="6" t="n">
+        <v>173</v>
+      </c>
+      <c r="F133" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-09-23 07:23 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1479,7 +1479,11 @@
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
-      <c r="C96" s="3" t="n"/>
+      <c r="C96" s="9" t="inlineStr">
+        <is>
+          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -1941,11 +1945,7 @@
           <t>d396b80a78fcbfbb48a9a68e42d5229d71a947bca970a9ccb07ba181250ab2d7</t>
         </is>
       </c>
-      <c r="C134" s="9" t="inlineStr">
-        <is>
-          <t>d396b80a78fcbfbb48a9a68e42d5229d71a947bca970a9ccb07ba181250ab2d7</t>
-        </is>
-      </c>
+      <c r="C134" s="3" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -2424,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F133"/>
+  <dimension ref="A1:F134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5631,6 +5631,30 @@
         </is>
       </c>
     </row>
+    <row r="134">
+      <c r="A134" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-23 07:13:39</t>
+        </is>
+      </c>
+      <c r="B134" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C134" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D134" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E134" s="5" t="n">
+        <v>173</v>
+      </c>
+      <c r="F134" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-09-24 07:07 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,11 +1366,7 @@
           <t>2f510140dc68e0c74c5ac10571c7237154c98f6810ad4b314bd1b1fedd391d49</t>
         </is>
       </c>
-      <c r="C87" s="9" t="inlineStr">
-        <is>
-          <t>2f510140dc68e0c74c5ac10571c7237154c98f6810ad4b314bd1b1fedd391d49</t>
-        </is>
-      </c>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1435,7 +1431,11 @@
           <t>ef692a6abff59e8b699d3e69d6974057ed5a5cc33d9d7a8f1d43f9f6342941f4</t>
         </is>
       </c>
-      <c r="C92" s="3" t="n"/>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
+          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -1479,11 +1479,7 @@
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
-      <c r="C96" s="9" t="inlineStr">
-        <is>
-          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
-        </is>
-      </c>
+      <c r="C96" s="3" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -2424,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F134"/>
+  <dimension ref="A1:F135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5655,6 +5651,30 @@
         </is>
       </c>
     </row>
+    <row r="135">
+      <c r="A135" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-24 07:05:41</t>
+        </is>
+      </c>
+      <c r="B135" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C135" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D135" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E135" s="6" t="n">
+        <v>174</v>
+      </c>
+      <c r="F135" s="6" t="inlineStr">
+        <is>
+          <t>PRM_AK_DHSS_EPL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-09-25 07:13 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,7 +1366,11 @@
           <t>2f510140dc68e0c74c5ac10571c7237154c98f6810ad4b314bd1b1fedd391d49</t>
         </is>
       </c>
-      <c r="C87" s="3" t="n"/>
+      <c r="C87" s="9" t="inlineStr">
+        <is>
+          <t>2f510140dc68e0c74c5ac10571c7237154c98f6810ad4b314bd1b1fedd391d49</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1428,14 +1432,10 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>ef692a6abff59e8b699d3e69d6974057ed5a5cc33d9d7a8f1d43f9f6342941f4</t>
-        </is>
-      </c>
-      <c r="C92" s="8" t="inlineStr">
-        <is>
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
+      <c r="C92" s="3" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -2420,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F135"/>
+  <dimension ref="A1:F136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5675,6 +5675,30 @@
         </is>
       </c>
     </row>
+    <row r="136">
+      <c r="A136" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-25 07:03:00</t>
+        </is>
+      </c>
+      <c r="B136" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C136" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D136" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E136" s="5" t="n">
+        <v>174</v>
+      </c>
+      <c r="F136" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-09-26 07:10 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,9 +1366,9 @@
           <t>2f510140dc68e0c74c5ac10571c7237154c98f6810ad4b314bd1b1fedd391d49</t>
         </is>
       </c>
-      <c r="C87" s="9" t="inlineStr">
-        <is>
-          <t>2f510140dc68e0c74c5ac10571c7237154c98f6810ad4b314bd1b1fedd391d49</t>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>1bf50fd27d84ee51530473c67ed01af779806dccbdbfaef9f8a6ab181dacaf88</t>
         </is>
       </c>
     </row>
@@ -1435,7 +1435,11 @@
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
-      <c r="C92" s="3" t="n"/>
+      <c r="C92" s="9" t="inlineStr">
+        <is>
+          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -2420,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F136"/>
+  <dimension ref="A1:F137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5699,6 +5703,30 @@
         </is>
       </c>
     </row>
+    <row r="137">
+      <c r="A137" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-26 07:00:07</t>
+        </is>
+      </c>
+      <c r="B137" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C137" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D137" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E137" s="6" t="n">
+        <v>173</v>
+      </c>
+      <c r="F137" s="6" t="inlineStr">
+        <is>
+          <t>OIG_MOST_WANTED</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-09-27 07:31 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1363,14 +1363,10 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>2f510140dc68e0c74c5ac10571c7237154c98f6810ad4b314bd1b1fedd391d49</t>
-        </is>
-      </c>
-      <c r="C87" s="8" t="inlineStr">
-        <is>
           <t>1bf50fd27d84ee51530473c67ed01af779806dccbdbfaef9f8a6ab181dacaf88</t>
         </is>
       </c>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1435,9 +1431,9 @@
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
-      <c r="C92" s="9" t="inlineStr">
-        <is>
-          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
+          <t>1bf50fd27d84ee51530473c67ed01af779806dccbdbfaef9f8a6ab181dacaf88</t>
         </is>
       </c>
     </row>
@@ -2261,7 +2257,11 @@
           <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
         </is>
       </c>
-      <c r="C162" s="3" t="n"/>
+      <c r="C162" s="8" t="inlineStr">
+        <is>
+          <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2424,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F137"/>
+  <dimension ref="A1:F138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5727,6 +5727,30 @@
         </is>
       </c>
     </row>
+    <row r="138">
+      <c r="A138" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-27 07:30:28</t>
+        </is>
+      </c>
+      <c r="B138" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C138" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D138" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E138" s="5" t="n">
+        <v>173</v>
+      </c>
+      <c r="F138" s="5" t="inlineStr">
+        <is>
+          <t>PRM_AK_DHSS_EPL, US_DOT_MOST_WANTED</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-09-28 08:18 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1428,10 +1428,10 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
-        </is>
-      </c>
-      <c r="C92" s="8" t="inlineStr">
+          <t>1bf50fd27d84ee51530473c67ed01af779806dccbdbfaef9f8a6ab181dacaf88</t>
+        </is>
+      </c>
+      <c r="C92" s="9" t="inlineStr">
         <is>
           <t>1bf50fd27d84ee51530473c67ed01af779806dccbdbfaef9f8a6ab181dacaf88</t>
         </is>
@@ -1479,7 +1479,11 @@
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
-      <c r="C96" s="3" t="n"/>
+      <c r="C96" s="9" t="inlineStr">
+        <is>
+          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -2254,14 +2258,10 @@
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>f871071363284514472663e563c727a9d4ec90158941ad2a970ab65fbe219806</t>
-        </is>
-      </c>
-      <c r="C162" s="8" t="inlineStr">
-        <is>
           <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
         </is>
       </c>
+      <c r="C162" s="3" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2424,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F138"/>
+  <dimension ref="A1:F139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5751,6 +5751,30 @@
         </is>
       </c>
     </row>
+    <row r="139">
+      <c r="A139" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-28 08:08:22</t>
+        </is>
+      </c>
+      <c r="B139" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C139" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D139" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E139" s="6" t="n">
+        <v>173</v>
+      </c>
+      <c r="F139" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-09-29 07:58 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,7 +1366,11 @@
           <t>1bf50fd27d84ee51530473c67ed01af779806dccbdbfaef9f8a6ab181dacaf88</t>
         </is>
       </c>
-      <c r="C87" s="3" t="n"/>
+      <c r="C87" s="9" t="inlineStr">
+        <is>
+          <t>1bf50fd27d84ee51530473c67ed01af779806dccbdbfaef9f8a6ab181dacaf88</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1431,11 +1435,7 @@
           <t>1bf50fd27d84ee51530473c67ed01af779806dccbdbfaef9f8a6ab181dacaf88</t>
         </is>
       </c>
-      <c r="C92" s="9" t="inlineStr">
-        <is>
-          <t>1bf50fd27d84ee51530473c67ed01af779806dccbdbfaef9f8a6ab181dacaf88</t>
-        </is>
-      </c>
+      <c r="C92" s="3" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -1479,11 +1479,7 @@
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
-      <c r="C96" s="9" t="inlineStr">
-        <is>
-          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
-        </is>
-      </c>
+      <c r="C96" s="3" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -2424,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F139"/>
+  <dimension ref="A1:F140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5775,6 +5771,30 @@
         </is>
       </c>
     </row>
+    <row r="140">
+      <c r="A140" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:48:47</t>
+        </is>
+      </c>
+      <c r="B140" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C140" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D140" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E140" s="5" t="n">
+        <v>174</v>
+      </c>
+      <c r="F140" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-09-30 08:02 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,11 +1366,7 @@
           <t>1bf50fd27d84ee51530473c67ed01af779806dccbdbfaef9f8a6ab181dacaf88</t>
         </is>
       </c>
-      <c r="C87" s="9" t="inlineStr">
-        <is>
-          <t>1bf50fd27d84ee51530473c67ed01af779806dccbdbfaef9f8a6ab181dacaf88</t>
-        </is>
-      </c>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -2420,7 +2416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F140"/>
+  <dimension ref="A1:F141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5795,6 +5791,30 @@
         </is>
       </c>
     </row>
+    <row r="141">
+      <c r="A141" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-30 07:51:53</t>
+        </is>
+      </c>
+      <c r="B141" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C141" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D141" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E141" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="F141" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-10-01 08:15 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -2253,7 +2253,11 @@
           <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
         </is>
       </c>
-      <c r="C162" s="3" t="n"/>
+      <c r="C162" s="8" t="inlineStr">
+        <is>
+          <t>52f25cfcb7477890bc538de42134463d2680432f99897039896b9eaed02dc225</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2416,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F141"/>
+  <dimension ref="A1:F142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5815,6 +5819,30 @@
         </is>
       </c>
     </row>
+    <row r="142">
+      <c r="A142" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-01 08:13:38</t>
+        </is>
+      </c>
+      <c r="B142" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C142" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D142" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E142" s="5" t="n">
+        <v>174</v>
+      </c>
+      <c r="F142" s="5" t="inlineStr">
+        <is>
+          <t>US_DOT_MOST_WANTED</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-10-02 07:54 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1937,7 +1937,11 @@
           <t>d396b80a78fcbfbb48a9a68e42d5229d71a947bca970a9ccb07ba181250ab2d7</t>
         </is>
       </c>
-      <c r="C134" s="3" t="n"/>
+      <c r="C134" s="9" t="inlineStr">
+        <is>
+          <t>d396b80a78fcbfbb48a9a68e42d5229d71a947bca970a9ccb07ba181250ab2d7</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -2250,14 +2254,10 @@
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
-        </is>
-      </c>
-      <c r="C162" s="8" t="inlineStr">
-        <is>
           <t>52f25cfcb7477890bc538de42134463d2680432f99897039896b9eaed02dc225</t>
         </is>
       </c>
+      <c r="C162" s="3" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2420,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F142"/>
+  <dimension ref="A1:F143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5843,6 +5843,30 @@
         </is>
       </c>
     </row>
+    <row r="143">
+      <c r="A143" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-02 07:52:33</t>
+        </is>
+      </c>
+      <c r="B143" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C143" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D143" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E143" s="6" t="n">
+        <v>174</v>
+      </c>
+      <c r="F143" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-10-03 07:31 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1937,11 +1937,7 @@
           <t>d396b80a78fcbfbb48a9a68e42d5229d71a947bca970a9ccb07ba181250ab2d7</t>
         </is>
       </c>
-      <c r="C134" s="9" t="inlineStr">
-        <is>
-          <t>d396b80a78fcbfbb48a9a68e42d5229d71a947bca970a9ccb07ba181250ab2d7</t>
-        </is>
-      </c>
+      <c r="C134" s="3" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -2257,7 +2253,11 @@
           <t>52f25cfcb7477890bc538de42134463d2680432f99897039896b9eaed02dc225</t>
         </is>
       </c>
-      <c r="C162" s="3" t="n"/>
+      <c r="C162" s="8" t="inlineStr">
+        <is>
+          <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2420,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F143"/>
+  <dimension ref="A1:F144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5867,6 +5867,30 @@
         </is>
       </c>
     </row>
+    <row r="144">
+      <c r="A144" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-03 07:30:01</t>
+        </is>
+      </c>
+      <c r="B144" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C144" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D144" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E144" s="5" t="n">
+        <v>174</v>
+      </c>
+      <c r="F144" s="5" t="inlineStr">
+        <is>
+          <t>US_DOT_MOST_WANTED</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-10-04 07:43 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1431,7 +1431,11 @@
           <t>1bf50fd27d84ee51530473c67ed01af779806dccbdbfaef9f8a6ab181dacaf88</t>
         </is>
       </c>
-      <c r="C92" s="3" t="n"/>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
+          <t>77f37815b610f4801760ca3422e8f1cce6377631a1b61a0c0465238f992ef286</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -2250,14 +2254,10 @@
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>52f25cfcb7477890bc538de42134463d2680432f99897039896b9eaed02dc225</t>
-        </is>
-      </c>
-      <c r="C162" s="8" t="inlineStr">
-        <is>
           <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
         </is>
       </c>
+      <c r="C162" s="3" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2420,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F144"/>
+  <dimension ref="A1:F145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5891,6 +5891,30 @@
         </is>
       </c>
     </row>
+    <row r="145">
+      <c r="A145" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-04 07:41:59</t>
+        </is>
+      </c>
+      <c r="B145" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C145" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D145" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E145" s="6" t="n">
+        <v>174</v>
+      </c>
+      <c r="F145" s="6" t="inlineStr">
+        <is>
+          <t>PRM_AK_DHSS_EPL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-10-05 08:12 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,7 +1366,11 @@
           <t>1bf50fd27d84ee51530473c67ed01af779806dccbdbfaef9f8a6ab181dacaf88</t>
         </is>
       </c>
-      <c r="C87" s="3" t="n"/>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>77f37815b610f4801760ca3422e8f1cce6377631a1b61a0c0465238f992ef286</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1428,12 +1432,12 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>1bf50fd27d84ee51530473c67ed01af779806dccbdbfaef9f8a6ab181dacaf88</t>
+          <t>77f37815b610f4801760ca3422e8f1cce6377631a1b61a0c0465238f992ef286</t>
         </is>
       </c>
       <c r="C92" s="8" t="inlineStr">
         <is>
-          <t>77f37815b610f4801760ca3422e8f1cce6377631a1b61a0c0465238f992ef286</t>
+          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
     </row>
@@ -2420,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F145"/>
+  <dimension ref="A1:F146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5915,6 +5919,30 @@
         </is>
       </c>
     </row>
+    <row r="146">
+      <c r="A146" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-05 08:10:53</t>
+        </is>
+      </c>
+      <c r="B146" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C146" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D146" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E146" s="5" t="n">
+        <v>173</v>
+      </c>
+      <c r="F146" s="5" t="inlineStr">
+        <is>
+          <t>OIG_MOST_WANTED, PRM_AK_DHSS_EPL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-10-06 08:39 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1363,10 +1363,10 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>1bf50fd27d84ee51530473c67ed01af779806dccbdbfaef9f8a6ab181dacaf88</t>
-        </is>
-      </c>
-      <c r="C87" s="8" t="inlineStr">
+          <t>77f37815b610f4801760ca3422e8f1cce6377631a1b61a0c0465238f992ef286</t>
+        </is>
+      </c>
+      <c r="C87" s="9" t="inlineStr">
         <is>
           <t>77f37815b610f4801760ca3422e8f1cce6377631a1b61a0c0465238f992ef286</t>
         </is>
@@ -1432,10 +1432,10 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>77f37815b610f4801760ca3422e8f1cce6377631a1b61a0c0465238f992ef286</t>
-        </is>
-      </c>
-      <c r="C92" s="8" t="inlineStr">
+          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
+        </is>
+      </c>
+      <c r="C92" s="9" t="inlineStr">
         <is>
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
@@ -2424,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F146"/>
+  <dimension ref="A1:F147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5943,6 +5943,30 @@
         </is>
       </c>
     </row>
+    <row r="147">
+      <c r="A147" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-06 08:29:10</t>
+        </is>
+      </c>
+      <c r="B147" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C147" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D147" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E147" s="6" t="n">
+        <v>173</v>
+      </c>
+      <c r="F147" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-10-07 08:06 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1435,11 +1435,7 @@
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
-      <c r="C92" s="9" t="inlineStr">
-        <is>
-          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
-        </is>
-      </c>
+      <c r="C92" s="3" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -2424,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F147"/>
+  <dimension ref="A1:F148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5967,6 +5963,30 @@
         </is>
       </c>
     </row>
+    <row r="148">
+      <c r="A148" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-07 08:04:36</t>
+        </is>
+      </c>
+      <c r="B148" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C148" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D148" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E148" s="5" t="n">
+        <v>174</v>
+      </c>
+      <c r="F148" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-10-08 08:22 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1941,7 +1941,11 @@
           <t>d396b80a78fcbfbb48a9a68e42d5229d71a947bca970a9ccb07ba181250ab2d7</t>
         </is>
       </c>
-      <c r="C134" s="3" t="n"/>
+      <c r="C134" s="9" t="inlineStr">
+        <is>
+          <t>d396b80a78fcbfbb48a9a68e42d5229d71a947bca970a9ccb07ba181250ab2d7</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -2257,7 +2261,11 @@
           <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
         </is>
       </c>
-      <c r="C162" s="3" t="n"/>
+      <c r="C162" s="9" t="inlineStr">
+        <is>
+          <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2420,7 +2428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F148"/>
+  <dimension ref="A1:F149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5987,6 +5995,30 @@
         </is>
       </c>
     </row>
+    <row r="149">
+      <c r="A149" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-08 08:21:11</t>
+        </is>
+      </c>
+      <c r="B149" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C149" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D149" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E149" s="6" t="n">
+        <v>172</v>
+      </c>
+      <c r="F149" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-10-09 08:25 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,11 +1366,7 @@
           <t>77f37815b610f4801760ca3422e8f1cce6377631a1b61a0c0465238f992ef286</t>
         </is>
       </c>
-      <c r="C87" s="9" t="inlineStr">
-        <is>
-          <t>77f37815b610f4801760ca3422e8f1cce6377631a1b61a0c0465238f992ef286</t>
-        </is>
-      </c>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1479,7 +1475,11 @@
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
-      <c r="C96" s="3" t="n"/>
+      <c r="C96" s="9" t="inlineStr">
+        <is>
+          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -2261,11 +2261,7 @@
           <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
         </is>
       </c>
-      <c r="C162" s="9" t="inlineStr">
-        <is>
-          <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
-        </is>
-      </c>
+      <c r="C162" s="3" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2428,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F149"/>
+  <dimension ref="A1:F150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6019,6 +6015,30 @@
         </is>
       </c>
     </row>
+    <row r="150">
+      <c r="A150" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-09 08:23:38</t>
+        </is>
+      </c>
+      <c r="B150" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C150" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D150" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E150" s="5" t="n">
+        <v>173</v>
+      </c>
+      <c r="F150" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-10-10 08:11 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,7 +1366,11 @@
           <t>77f37815b610f4801760ca3422e8f1cce6377631a1b61a0c0465238f992ef286</t>
         </is>
       </c>
-      <c r="C87" s="3" t="n"/>
+      <c r="C87" s="9" t="inlineStr">
+        <is>
+          <t>77f37815b610f4801760ca3422e8f1cce6377631a1b61a0c0465238f992ef286</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1475,11 +1479,7 @@
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
-      <c r="C96" s="9" t="inlineStr">
-        <is>
-          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
-        </is>
-      </c>
+      <c r="C96" s="3" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -1941,11 +1941,7 @@
           <t>d396b80a78fcbfbb48a9a68e42d5229d71a947bca970a9ccb07ba181250ab2d7</t>
         </is>
       </c>
-      <c r="C134" s="9" t="inlineStr">
-        <is>
-          <t>d396b80a78fcbfbb48a9a68e42d5229d71a947bca970a9ccb07ba181250ab2d7</t>
-        </is>
-      </c>
+      <c r="C134" s="3" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -2424,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F150"/>
+  <dimension ref="A1:F151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6039,6 +6035,30 @@
         </is>
       </c>
     </row>
+    <row r="151">
+      <c r="A151" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-10 08:00:54</t>
+        </is>
+      </c>
+      <c r="B151" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C151" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D151" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E151" s="6" t="n">
+        <v>174</v>
+      </c>
+      <c r="F151" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-10-11 08:14 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,11 +1366,7 @@
           <t>77f37815b610f4801760ca3422e8f1cce6377631a1b61a0c0465238f992ef286</t>
         </is>
       </c>
-      <c r="C87" s="9" t="inlineStr">
-        <is>
-          <t>77f37815b610f4801760ca3422e8f1cce6377631a1b61a0c0465238f992ef286</t>
-        </is>
-      </c>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1435,7 +1431,11 @@
           <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
         </is>
       </c>
-      <c r="C92" s="3" t="n"/>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
+          <t>77f37815b610f4801760ca3422e8f1cce6377631a1b61a0c0465238f992ef286</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -1941,7 +1941,11 @@
           <t>d396b80a78fcbfbb48a9a68e42d5229d71a947bca970a9ccb07ba181250ab2d7</t>
         </is>
       </c>
-      <c r="C134" s="3" t="n"/>
+      <c r="C134" s="9" t="inlineStr">
+        <is>
+          <t>d396b80a78fcbfbb48a9a68e42d5229d71a947bca970a9ccb07ba181250ab2d7</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -2420,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F151"/>
+  <dimension ref="A1:F152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6059,6 +6063,30 @@
         </is>
       </c>
     </row>
+    <row r="152">
+      <c r="A152" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-11 08:12:50</t>
+        </is>
+      </c>
+      <c r="B152" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C152" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D152" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E152" s="5" t="n">
+        <v>173</v>
+      </c>
+      <c r="F152" s="5" t="inlineStr">
+        <is>
+          <t>PRM_AK_DHSS_EPL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-10-12 08:39 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,7 +1366,11 @@
           <t>77f37815b610f4801760ca3422e8f1cce6377631a1b61a0c0465238f992ef286</t>
         </is>
       </c>
-      <c r="C87" s="3" t="n"/>
+      <c r="C87" s="9" t="inlineStr">
+        <is>
+          <t>77f37815b610f4801760ca3422e8f1cce6377631a1b61a0c0465238f992ef286</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1428,12 +1432,12 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>5b10138af207dad51d825b32199e50cb6a6d5138533b41c17ce98bcb85040325</t>
+          <t>77f37815b610f4801760ca3422e8f1cce6377631a1b61a0c0465238f992ef286</t>
         </is>
       </c>
       <c r="C92" s="8" t="inlineStr">
         <is>
-          <t>77f37815b610f4801760ca3422e8f1cce6377631a1b61a0c0465238f992ef286</t>
+          <t>c3544f17959b207b14f0514baf96ecc4adefed6349ea27b6e250a2209b717832</t>
         </is>
       </c>
     </row>
@@ -1941,11 +1945,7 @@
           <t>d396b80a78fcbfbb48a9a68e42d5229d71a947bca970a9ccb07ba181250ab2d7</t>
         </is>
       </c>
-      <c r="C134" s="9" t="inlineStr">
-        <is>
-          <t>d396b80a78fcbfbb48a9a68e42d5229d71a947bca970a9ccb07ba181250ab2d7</t>
-        </is>
-      </c>
+      <c r="C134" s="3" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -2424,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F152"/>
+  <dimension ref="A1:F153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6087,6 +6087,30 @@
         </is>
       </c>
     </row>
+    <row r="153">
+      <c r="A153" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-12 08:29:16</t>
+        </is>
+      </c>
+      <c r="B153" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C153" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D153" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E153" s="6" t="n">
+        <v>173</v>
+      </c>
+      <c r="F153" s="6" t="inlineStr">
+        <is>
+          <t>PRM_AK_DHSS_EPL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-10-13 08:54 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1432,14 +1432,10 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>77f37815b610f4801760ca3422e8f1cce6377631a1b61a0c0465238f992ef286</t>
-        </is>
-      </c>
-      <c r="C92" s="8" t="inlineStr">
-        <is>
           <t>c3544f17959b207b14f0514baf96ecc4adefed6349ea27b6e250a2209b717832</t>
         </is>
       </c>
+      <c r="C92" s="3" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -1483,7 +1479,11 @@
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
-      <c r="C96" s="3" t="n"/>
+      <c r="C96" s="9" t="inlineStr">
+        <is>
+          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -1945,7 +1945,11 @@
           <t>d396b80a78fcbfbb48a9a68e42d5229d71a947bca970a9ccb07ba181250ab2d7</t>
         </is>
       </c>
-      <c r="C134" s="3" t="n"/>
+      <c r="C134" s="8" t="inlineStr">
+        <is>
+          <t>6976a74b56d44cad0a67a0885d32918bf0a613d8d6a446d3b5490f476a3f7ac1</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -2424,7 +2428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F153"/>
+  <dimension ref="A1:F154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6111,6 +6115,30 @@
         </is>
       </c>
     </row>
+    <row r="154">
+      <c r="A154" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13 08:52:32</t>
+        </is>
+      </c>
+      <c r="B154" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C154" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D154" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E154" s="5" t="n">
+        <v>172</v>
+      </c>
+      <c r="F154" s="5" t="inlineStr">
+        <is>
+          <t>PRM_WI_DOT_DSIC</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-10-14 07:03 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,11 +1366,7 @@
           <t>77f37815b610f4801760ca3422e8f1cce6377631a1b61a0c0465238f992ef286</t>
         </is>
       </c>
-      <c r="C87" s="9" t="inlineStr">
-        <is>
-          <t>77f37815b610f4801760ca3422e8f1cce6377631a1b61a0c0465238f992ef286</t>
-        </is>
-      </c>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1435,7 +1431,11 @@
           <t>c3544f17959b207b14f0514baf96ecc4adefed6349ea27b6e250a2209b717832</t>
         </is>
       </c>
-      <c r="C92" s="3" t="n"/>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
+          <t>77f37815b610f4801760ca3422e8f1cce6377631a1b61a0c0465238f992ef286</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -1479,11 +1479,7 @@
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
-      <c r="C96" s="9" t="inlineStr">
-        <is>
-          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
-        </is>
-      </c>
+      <c r="C96" s="3" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -1942,10 +1938,10 @@
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>d396b80a78fcbfbb48a9a68e42d5229d71a947bca970a9ccb07ba181250ab2d7</t>
-        </is>
-      </c>
-      <c r="C134" s="8" t="inlineStr">
+          <t>6976a74b56d44cad0a67a0885d32918bf0a613d8d6a446d3b5490f476a3f7ac1</t>
+        </is>
+      </c>
+      <c r="C134" s="9" t="inlineStr">
         <is>
           <t>6976a74b56d44cad0a67a0885d32918bf0a613d8d6a446d3b5490f476a3f7ac1</t>
         </is>
@@ -2428,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F154"/>
+  <dimension ref="A1:F155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6139,6 +6135,30 @@
         </is>
       </c>
     </row>
+    <row r="155">
+      <c r="A155" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14 07:02:31</t>
+        </is>
+      </c>
+      <c r="B155" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C155" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D155" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E155" s="6" t="n">
+        <v>173</v>
+      </c>
+      <c r="F155" s="6" t="inlineStr">
+        <is>
+          <t>PRM_AK_DHSS_EPL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-10-15 06:55 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1428,12 +1428,12 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>c3544f17959b207b14f0514baf96ecc4adefed6349ea27b6e250a2209b717832</t>
+          <t>77f37815b610f4801760ca3422e8f1cce6377631a1b61a0c0465238f992ef286</t>
         </is>
       </c>
       <c r="C92" s="8" t="inlineStr">
         <is>
-          <t>77f37815b610f4801760ca3422e8f1cce6377631a1b61a0c0465238f992ef286</t>
+          <t>257e819d07de9a7ac8a90a0e0c1ffef572a7b5d2baf096df74fd8f3c9e608e53</t>
         </is>
       </c>
     </row>
@@ -2424,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F155"/>
+  <dimension ref="A1:F156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6159,6 +6159,30 @@
         </is>
       </c>
     </row>
+    <row r="156">
+      <c r="A156" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-15 06:53:33</t>
+        </is>
+      </c>
+      <c r="B156" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C156" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D156" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E156" s="5" t="n">
+        <v>173</v>
+      </c>
+      <c r="F156" s="5" t="inlineStr">
+        <is>
+          <t>PRM_AK_DHSS_EPL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-10-16 06:42 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1428,14 +1428,10 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>77f37815b610f4801760ca3422e8f1cce6377631a1b61a0c0465238f992ef286</t>
-        </is>
-      </c>
-      <c r="C92" s="8" t="inlineStr">
-        <is>
           <t>257e819d07de9a7ac8a90a0e0c1ffef572a7b5d2baf096df74fd8f3c9e608e53</t>
         </is>
       </c>
+      <c r="C92" s="3" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -1479,7 +1475,11 @@
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
-      <c r="C96" s="3" t="n"/>
+      <c r="C96" s="8" t="inlineStr">
+        <is>
+          <t>c3544f17959b207b14f0514baf96ecc4adefed6349ea27b6e250a2209b717832</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -2424,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F156"/>
+  <dimension ref="A1:F157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6183,6 +6183,30 @@
         </is>
       </c>
     </row>
+    <row r="157">
+      <c r="A157" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-16 06:40:51</t>
+        </is>
+      </c>
+      <c r="B157" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C157" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D157" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E157" s="6" t="n">
+        <v>173</v>
+      </c>
+      <c r="F157" s="6" t="inlineStr">
+        <is>
+          <t>PRM_CA_DIR_DC</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-10-17 06:39 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1472,14 +1472,10 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
-        </is>
-      </c>
-      <c r="C96" s="8" t="inlineStr">
-        <is>
           <t>c3544f17959b207b14f0514baf96ecc4adefed6349ea27b6e250a2209b717832</t>
         </is>
       </c>
+      <c r="C96" s="3" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -1941,11 +1937,7 @@
           <t>6976a74b56d44cad0a67a0885d32918bf0a613d8d6a446d3b5490f476a3f7ac1</t>
         </is>
       </c>
-      <c r="C134" s="9" t="inlineStr">
-        <is>
-          <t>6976a74b56d44cad0a67a0885d32918bf0a613d8d6a446d3b5490f476a3f7ac1</t>
-        </is>
-      </c>
+      <c r="C134" s="3" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -2424,7 +2416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F157"/>
+  <dimension ref="A1:F158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6207,6 +6199,30 @@
         </is>
       </c>
     </row>
+    <row r="158">
+      <c r="A158" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-17 06:29:39</t>
+        </is>
+      </c>
+      <c r="B158" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C158" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D158" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E158" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="F158" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-10-18 07:04 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,7 +1366,11 @@
           <t>77f37815b610f4801760ca3422e8f1cce6377631a1b61a0c0465238f992ef286</t>
         </is>
       </c>
-      <c r="C87" s="3" t="n"/>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>c1803870b5a3e4b3bec257cf479dbe8b139fb9c54f269a9c91df3dbedb3c077f</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1431,7 +1435,11 @@
           <t>257e819d07de9a7ac8a90a0e0c1ffef572a7b5d2baf096df74fd8f3c9e608e53</t>
         </is>
       </c>
-      <c r="C92" s="3" t="n"/>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
+          <t>c3544f17959b207b14f0514baf96ecc4adefed6349ea27b6e250a2209b717832</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -2337,7 +2345,11 @@
           <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
         </is>
       </c>
-      <c r="C170" s="3" t="n"/>
+      <c r="C170" s="8" t="inlineStr">
+        <is>
+          <t>52f25cfcb7477890bc538de42134463d2680432f99897039896b9eaed02dc225</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -2416,7 +2428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F158"/>
+  <dimension ref="A1:F159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6223,6 +6235,30 @@
         </is>
       </c>
     </row>
+    <row r="159">
+      <c r="A159" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-18 06:54:42</t>
+        </is>
+      </c>
+      <c r="B159" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C159" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D159" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E159" s="6" t="n">
+        <v>172</v>
+      </c>
+      <c r="F159" s="6" t="inlineStr">
+        <is>
+          <t>OIG_MOST_WANTED, PRM_AK_DHSS_EPL, US_PDGS_IFP_LIST</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-10-19 07:15 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1363,14 +1363,10 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>77f37815b610f4801760ca3422e8f1cce6377631a1b61a0c0465238f992ef286</t>
-        </is>
-      </c>
-      <c r="C87" s="8" t="inlineStr">
-        <is>
           <t>c1803870b5a3e4b3bec257cf479dbe8b139fb9c54f269a9c91df3dbedb3c077f</t>
         </is>
       </c>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1432,14 +1428,10 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>257e819d07de9a7ac8a90a0e0c1ffef572a7b5d2baf096df74fd8f3c9e608e53</t>
-        </is>
-      </c>
-      <c r="C92" s="8" t="inlineStr">
-        <is>
           <t>c3544f17959b207b14f0514baf96ecc4adefed6349ea27b6e250a2209b717832</t>
         </is>
       </c>
+      <c r="C92" s="3" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -2342,14 +2334,10 @@
       </c>
       <c r="B170" s="2" t="inlineStr">
         <is>
-          <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
-        </is>
-      </c>
-      <c r="C170" s="8" t="inlineStr">
-        <is>
           <t>52f25cfcb7477890bc538de42134463d2680432f99897039896b9eaed02dc225</t>
         </is>
       </c>
+      <c r="C170" s="3" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -2428,7 +2416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F159"/>
+  <dimension ref="A1:F160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6259,6 +6247,30 @@
         </is>
       </c>
     </row>
+    <row r="160">
+      <c r="A160" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-19 07:14:30</t>
+        </is>
+      </c>
+      <c r="B160" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C160" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D160" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E160" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="F160" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-10-20 07:04 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1475,7 +1475,11 @@
           <t>c3544f17959b207b14f0514baf96ecc4adefed6349ea27b6e250a2209b717832</t>
         </is>
       </c>
-      <c r="C96" s="3" t="n"/>
+      <c r="C96" s="8" t="inlineStr">
+        <is>
+          <t>c1803870b5a3e4b3bec257cf479dbe8b139fb9c54f269a9c91df3dbedb3c077f</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -2416,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F160"/>
+  <dimension ref="A1:F161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6271,6 +6275,30 @@
         </is>
       </c>
     </row>
+    <row r="161">
+      <c r="A161" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:03:15</t>
+        </is>
+      </c>
+      <c r="B161" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C161" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D161" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E161" s="6" t="n">
+        <v>174</v>
+      </c>
+      <c r="F161" s="6" t="inlineStr">
+        <is>
+          <t>PRM_CA_DIR_DC</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-10-21 07:06 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,7 +1366,11 @@
           <t>c1803870b5a3e4b3bec257cf479dbe8b139fb9c54f269a9c91df3dbedb3c077f</t>
         </is>
       </c>
-      <c r="C87" s="3" t="n"/>
+      <c r="C87" s="9" t="inlineStr">
+        <is>
+          <t>c1803870b5a3e4b3bec257cf479dbe8b139fb9c54f269a9c91df3dbedb3c077f</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1472,14 +1476,10 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>c3544f17959b207b14f0514baf96ecc4adefed6349ea27b6e250a2209b717832</t>
-        </is>
-      </c>
-      <c r="C96" s="8" t="inlineStr">
-        <is>
           <t>c1803870b5a3e4b3bec257cf479dbe8b139fb9c54f269a9c91df3dbedb3c077f</t>
         </is>
       </c>
+      <c r="C96" s="3" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -2420,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F161"/>
+  <dimension ref="A1:F162"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6299,6 +6299,30 @@
         </is>
       </c>
     </row>
+    <row r="162">
+      <c r="A162" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-21 06:56:43</t>
+        </is>
+      </c>
+      <c r="B162" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C162" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D162" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E162" s="5" t="n">
+        <v>174</v>
+      </c>
+      <c r="F162" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-10-22 07:02 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,11 +1366,7 @@
           <t>c1803870b5a3e4b3bec257cf479dbe8b139fb9c54f269a9c91df3dbedb3c077f</t>
         </is>
       </c>
-      <c r="C87" s="9" t="inlineStr">
-        <is>
-          <t>c1803870b5a3e4b3bec257cf479dbe8b139fb9c54f269a9c91df3dbedb3c077f</t>
-        </is>
-      </c>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1941,7 +1937,11 @@
           <t>6976a74b56d44cad0a67a0885d32918bf0a613d8d6a446d3b5490f476a3f7ac1</t>
         </is>
       </c>
-      <c r="C134" s="3" t="n"/>
+      <c r="C134" s="9" t="inlineStr">
+        <is>
+          <t>6976a74b56d44cad0a67a0885d32918bf0a613d8d6a446d3b5490f476a3f7ac1</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -2420,7 +2420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F162"/>
+  <dimension ref="A1:F163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6323,6 +6323,30 @@
         </is>
       </c>
     </row>
+    <row r="163">
+      <c r="A163" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-22 07:00:54</t>
+        </is>
+      </c>
+      <c r="B163" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C163" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D163" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E163" s="6" t="n">
+        <v>174</v>
+      </c>
+      <c r="F163" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-10-23 07:03 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,7 +1366,11 @@
           <t>c1803870b5a3e4b3bec257cf479dbe8b139fb9c54f269a9c91df3dbedb3c077f</t>
         </is>
       </c>
-      <c r="C87" s="3" t="n"/>
+      <c r="C87" s="9" t="inlineStr">
+        <is>
+          <t>c1803870b5a3e4b3bec257cf479dbe8b139fb9c54f269a9c91df3dbedb3c077f</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1431,7 +1435,11 @@
           <t>c3544f17959b207b14f0514baf96ecc4adefed6349ea27b6e250a2209b717832</t>
         </is>
       </c>
-      <c r="C92" s="3" t="n"/>
+      <c r="C92" s="9" t="inlineStr">
+        <is>
+          <t>c3544f17959b207b14f0514baf96ecc4adefed6349ea27b6e250a2209b717832</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -1937,11 +1945,7 @@
           <t>6976a74b56d44cad0a67a0885d32918bf0a613d8d6a446d3b5490f476a3f7ac1</t>
         </is>
       </c>
-      <c r="C134" s="9" t="inlineStr">
-        <is>
-          <t>6976a74b56d44cad0a67a0885d32918bf0a613d8d6a446d3b5490f476a3f7ac1</t>
-        </is>
-      </c>
+      <c r="C134" s="3" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -2420,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F163"/>
+  <dimension ref="A1:F164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6347,6 +6351,30 @@
         </is>
       </c>
     </row>
+    <row r="164">
+      <c r="A164" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23 06:53:13</t>
+        </is>
+      </c>
+      <c r="B164" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C164" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D164" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E164" s="5" t="n">
+        <v>173</v>
+      </c>
+      <c r="F164" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-10-24 06:50 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,11 +1366,7 @@
           <t>c1803870b5a3e4b3bec257cf479dbe8b139fb9c54f269a9c91df3dbedb3c077f</t>
         </is>
       </c>
-      <c r="C87" s="9" t="inlineStr">
-        <is>
-          <t>c1803870b5a3e4b3bec257cf479dbe8b139fb9c54f269a9c91df3dbedb3c077f</t>
-        </is>
-      </c>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1435,9 +1431,9 @@
           <t>c3544f17959b207b14f0514baf96ecc4adefed6349ea27b6e250a2209b717832</t>
         </is>
       </c>
-      <c r="C92" s="9" t="inlineStr">
-        <is>
-          <t>c3544f17959b207b14f0514baf96ecc4adefed6349ea27b6e250a2209b717832</t>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
+          <t>c1803870b5a3e4b3bec257cf479dbe8b139fb9c54f269a9c91df3dbedb3c077f</t>
         </is>
       </c>
     </row>
@@ -1483,7 +1479,11 @@
           <t>c1803870b5a3e4b3bec257cf479dbe8b139fb9c54f269a9c91df3dbedb3c077f</t>
         </is>
       </c>
-      <c r="C96" s="3" t="n"/>
+      <c r="C96" s="8" t="inlineStr">
+        <is>
+          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -2424,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F164"/>
+  <dimension ref="A1:F165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6375,6 +6375,30 @@
         </is>
       </c>
     </row>
+    <row r="165">
+      <c r="A165" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-24 06:49:10</t>
+        </is>
+      </c>
+      <c r="B165" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C165" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D165" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E165" s="6" t="n">
+        <v>173</v>
+      </c>
+      <c r="F165" s="6" t="inlineStr">
+        <is>
+          <t>PRM_AK_DHSS_EPL, PRM_CA_DIR_DC</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-10-25 07:14 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1428,14 +1428,10 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>c3544f17959b207b14f0514baf96ecc4adefed6349ea27b6e250a2209b717832</t>
-        </is>
-      </c>
-      <c r="C92" s="8" t="inlineStr">
-        <is>
           <t>c1803870b5a3e4b3bec257cf479dbe8b139fb9c54f269a9c91df3dbedb3c077f</t>
         </is>
       </c>
+      <c r="C92" s="3" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -1476,14 +1472,10 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>c1803870b5a3e4b3bec257cf479dbe8b139fb9c54f269a9c91df3dbedb3c077f</t>
-        </is>
-      </c>
-      <c r="C96" s="8" t="inlineStr">
-        <is>
           <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
         </is>
       </c>
+      <c r="C96" s="3" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -2424,7 +2416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F165"/>
+  <dimension ref="A1:F166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6399,6 +6391,30 @@
         </is>
       </c>
     </row>
+    <row r="166">
+      <c r="A166" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-25 07:12:57</t>
+        </is>
+      </c>
+      <c r="B166" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C166" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D166" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E166" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="F166" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-10-26 07:23 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,7 +1366,11 @@
           <t>c1803870b5a3e4b3bec257cf479dbe8b139fb9c54f269a9c91df3dbedb3c077f</t>
         </is>
       </c>
-      <c r="C87" s="3" t="n"/>
+      <c r="C87" s="9" t="inlineStr">
+        <is>
+          <t>c1803870b5a3e4b3bec257cf479dbe8b139fb9c54f269a9c91df3dbedb3c077f</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1431,7 +1435,11 @@
           <t>c1803870b5a3e4b3bec257cf479dbe8b139fb9c54f269a9c91df3dbedb3c077f</t>
         </is>
       </c>
-      <c r="C92" s="3" t="n"/>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
+          <t>c3544f17959b207b14f0514baf96ecc4adefed6349ea27b6e250a2209b717832</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -1937,7 +1945,11 @@
           <t>6976a74b56d44cad0a67a0885d32918bf0a613d8d6a446d3b5490f476a3f7ac1</t>
         </is>
       </c>
-      <c r="C134" s="3" t="n"/>
+      <c r="C134" s="9" t="inlineStr">
+        <is>
+          <t>6976a74b56d44cad0a67a0885d32918bf0a613d8d6a446d3b5490f476a3f7ac1</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -2416,7 +2428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F166"/>
+  <dimension ref="A1:F167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6415,6 +6427,30 @@
         </is>
       </c>
     </row>
+    <row r="167">
+      <c r="A167" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-26 07:21:27</t>
+        </is>
+      </c>
+      <c r="B167" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C167" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D167" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E167" s="6" t="n">
+        <v>172</v>
+      </c>
+      <c r="F167" s="6" t="inlineStr">
+        <is>
+          <t>PRM_AK_DHSS_EPL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-10-27 07:14 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1432,14 +1432,10 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>c1803870b5a3e4b3bec257cf479dbe8b139fb9c54f269a9c91df3dbedb3c077f</t>
-        </is>
-      </c>
-      <c r="C92" s="8" t="inlineStr">
-        <is>
           <t>c3544f17959b207b14f0514baf96ecc4adefed6349ea27b6e250a2209b717832</t>
         </is>
       </c>
+      <c r="C92" s="3" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -2265,7 +2261,11 @@
           <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
         </is>
       </c>
-      <c r="C162" s="3" t="n"/>
+      <c r="C162" s="9" t="inlineStr">
+        <is>
+          <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2428,7 +2428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F167"/>
+  <dimension ref="A1:F168"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6451,6 +6451,30 @@
         </is>
       </c>
     </row>
+    <row r="168">
+      <c r="A168" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-27 07:12:47</t>
+        </is>
+      </c>
+      <c r="B168" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C168" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D168" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E168" s="5" t="n">
+        <v>172</v>
+      </c>
+      <c r="F168" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-10-28 08:02 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1941,11 +1941,7 @@
           <t>6976a74b56d44cad0a67a0885d32918bf0a613d8d6a446d3b5490f476a3f7ac1</t>
         </is>
       </c>
-      <c r="C134" s="9" t="inlineStr">
-        <is>
-          <t>6976a74b56d44cad0a67a0885d32918bf0a613d8d6a446d3b5490f476a3f7ac1</t>
-        </is>
-      </c>
+      <c r="C134" s="3" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -2428,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F168"/>
+  <dimension ref="A1:F169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6475,6 +6471,30 @@
         </is>
       </c>
     </row>
+    <row r="169">
+      <c r="A169" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-28 07:51:46</t>
+        </is>
+      </c>
+      <c r="B169" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C169" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D169" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E169" s="6" t="n">
+        <v>173</v>
+      </c>
+      <c r="F169" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-10-29 07:58 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1366,11 +1366,7 @@
           <t>c1803870b5a3e4b3bec257cf479dbe8b139fb9c54f269a9c91df3dbedb3c077f</t>
         </is>
       </c>
-      <c r="C87" s="9" t="inlineStr">
-        <is>
-          <t>c1803870b5a3e4b3bec257cf479dbe8b139fb9c54f269a9c91df3dbedb3c077f</t>
-        </is>
-      </c>
+      <c r="C87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1435,7 +1431,11 @@
           <t>c3544f17959b207b14f0514baf96ecc4adefed6349ea27b6e250a2209b717832</t>
         </is>
       </c>
-      <c r="C92" s="3" t="n"/>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
+          <t>e2e7727dac83eac54b743db9748099b2cdace93aceb1e32d1609109b050588fc</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -1941,7 +1941,11 @@
           <t>6976a74b56d44cad0a67a0885d32918bf0a613d8d6a446d3b5490f476a3f7ac1</t>
         </is>
       </c>
-      <c r="C134" s="3" t="n"/>
+      <c r="C134" s="9" t="inlineStr">
+        <is>
+          <t>6976a74b56d44cad0a67a0885d32918bf0a613d8d6a446d3b5490f476a3f7ac1</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -2257,11 +2261,7 @@
           <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
         </is>
       </c>
-      <c r="C162" s="9" t="inlineStr">
-        <is>
-          <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
-        </is>
-      </c>
+      <c r="C162" s="3" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2424,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F169"/>
+  <dimension ref="A1:F170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6495,6 +6495,30 @@
         </is>
       </c>
     </row>
+    <row r="170">
+      <c r="A170" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-29 07:57:17</t>
+        </is>
+      </c>
+      <c r="B170" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C170" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D170" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E170" s="5" t="n">
+        <v>173</v>
+      </c>
+      <c r="F170" s="5" t="inlineStr">
+        <is>
+          <t>PRM_AK_DHSS_EPL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-10-30 08:00 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1428,14 +1428,10 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>c3544f17959b207b14f0514baf96ecc4adefed6349ea27b6e250a2209b717832</t>
-        </is>
-      </c>
-      <c r="C92" s="8" t="inlineStr">
-        <is>
           <t>e2e7727dac83eac54b743db9748099b2cdace93aceb1e32d1609109b050588fc</t>
         </is>
       </c>
+      <c r="C92" s="3" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -2319,7 +2315,11 @@
           <t>52f25cfcb7477890bc538de42134463d2680432f99897039896b9eaed02dc225</t>
         </is>
       </c>
-      <c r="C168" s="3" t="n"/>
+      <c r="C168" s="8" t="inlineStr">
+        <is>
+          <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -2424,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F170"/>
+  <dimension ref="A1:F171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6519,6 +6519,30 @@
         </is>
       </c>
     </row>
+    <row r="171">
+      <c r="A171" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-30 07:59:30</t>
+        </is>
+      </c>
+      <c r="B171" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="C171" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D171" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E171" s="6" t="n">
+        <v>173</v>
+      </c>
+      <c r="F171" s="6" t="inlineStr">
+        <is>
+          <t>US_NJL_IDA</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update RPS hash values [2026-10-31 07:56 UTC]
</commit_message>
<xml_diff>
--- a/RPS_Updates.xlsx
+++ b/RPS_Updates.xlsx
@@ -1431,7 +1431,11 @@
           <t>e2e7727dac83eac54b743db9748099b2cdace93aceb1e32d1609109b050588fc</t>
         </is>
       </c>
-      <c r="C92" s="3" t="n"/>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
+          <t>85fc59fc5c4eab0d9f64c8713608aafb05cbe9d69a782410e6a65db0d42feb11</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -1937,11 +1941,7 @@
           <t>6976a74b56d44cad0a67a0885d32918bf0a613d8d6a446d3b5490f476a3f7ac1</t>
         </is>
       </c>
-      <c r="C134" s="9" t="inlineStr">
-        <is>
-          <t>6976a74b56d44cad0a67a0885d32918bf0a613d8d6a446d3b5490f476a3f7ac1</t>
-        </is>
-      </c>
+      <c r="C134" s="3" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -2257,7 +2257,11 @@
           <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
         </is>
       </c>
-      <c r="C162" s="3" t="n"/>
+      <c r="C162" s="9" t="inlineStr">
+        <is>
+          <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -2312,14 +2316,10 @@
       </c>
       <c r="B168" s="2" t="inlineStr">
         <is>
-          <t>52f25cfcb7477890bc538de42134463d2680432f99897039896b9eaed02dc225</t>
-        </is>
-      </c>
-      <c r="C168" s="8" t="inlineStr">
-        <is>
           <t>cd37a8abbd9b71a1acf19d4be7bace24d51c64de0eb54e3941ff77e78debac24</t>
         </is>
       </c>
+      <c r="C168" s="3" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -2424,7 +2424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F171"/>
+  <dimension ref="A1:F172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6543,6 +6543,30 @@
         </is>
       </c>
     </row>
+    <row r="172">
+      <c r="A172" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-31 07:55:31</t>
+        </is>
+      </c>
+      <c r="B172" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C172" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D172" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E172" s="5" t="n">
+        <v>173</v>
+      </c>
+      <c r="F172" s="5" t="inlineStr">
+        <is>
+          <t>PRM_AK_DHSS_EPL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>